<commit_message>
fix: record Sadang 17 union-establishment approval in Golden SoT
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/archive/golden/260823/golden_samples_260823.xlsx
+++ b/data/archive/golden/260823/golden_samples_260823.xlsx
@@ -3562,7 +3562,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>추진위 승인</t>
+          <t>조합설립인가</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>26년 1월 7일 추진위 승인</t>
+          <t>26년 8월 21일 조합설립인가</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3639,7 +3639,7 @@
 기획완료|2025.8.6
 추진위승인|2026.1.7
 정비구역지정|2026.1.22
-조합설립인가|6개월째 진행중(평균 14개월)</t>
+조합설립인가|2026.8.21</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">

</xml_diff>